<commit_message>
feat: update Excel template with new food market categories
- Master Data sheet: 200 rows ready
- Summary sheet: 16 categories with COUNTIF/SUMIF formulas

https://claude.ai/code/session_01Fs1HP51uTb2BEdsbuJ8DpT
</commit_message>
<xml_diff>
--- a/expense_tracker_template.xlsx
+++ b/expense_tracker_template.xlsx
@@ -503,11 +503,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
@@ -1058,6 +1058,1506 @@
       <c r="G51" s="4" t="inlineStr"/>
       <c r="H51" s="4" t="inlineStr"/>
     </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="4" t="inlineStr"/>
+      <c r="B53" s="4" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr"/>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
+      <c r="H53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="3" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr"/>
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="3" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="4" t="inlineStr"/>
+      <c r="B57" s="4" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="3" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="4" t="inlineStr"/>
+      <c r="B59" s="4" t="inlineStr"/>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="2" t="inlineStr"/>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="3" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="4" t="inlineStr"/>
+      <c r="B61" s="4" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="4" t="inlineStr"/>
+      <c r="B63" s="4" t="inlineStr"/>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="4" t="inlineStr"/>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="2" t="inlineStr"/>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="4" t="inlineStr"/>
+      <c r="B65" s="4" t="inlineStr"/>
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr"/>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="2" t="inlineStr"/>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="C66" s="3" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="4" t="inlineStr"/>
+      <c r="B67" s="4" t="inlineStr"/>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr"/>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="2" t="inlineStr"/>
+      <c r="B68" s="2" t="inlineStr"/>
+      <c r="C68" s="3" t="inlineStr"/>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="4" t="inlineStr"/>
+      <c r="B69" s="4" t="inlineStr"/>
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr"/>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr"/>
+      <c r="B70" s="2" t="inlineStr"/>
+      <c r="C70" s="3" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="4" t="inlineStr"/>
+      <c r="B71" s="4" t="inlineStr"/>
+      <c r="C71" s="5" t="inlineStr"/>
+      <c r="D71" s="4" t="inlineStr"/>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="inlineStr"/>
+      <c r="B72" s="2" t="inlineStr"/>
+      <c r="C72" s="3" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="inlineStr"/>
+      <c r="C73" s="5" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr"/>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr"/>
+      <c r="H73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="inlineStr"/>
+      <c r="B74" s="2" t="inlineStr"/>
+      <c r="C74" s="3" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="4" t="inlineStr"/>
+      <c r="B75" s="4" t="inlineStr"/>
+      <c r="C75" s="5" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr"/>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="inlineStr"/>
+      <c r="B76" s="2" t="inlineStr"/>
+      <c r="C76" s="3" t="inlineStr"/>
+      <c r="D76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="4" t="inlineStr"/>
+      <c r="B77" s="4" t="inlineStr"/>
+      <c r="C77" s="5" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr"/>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr"/>
+      <c r="H77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="inlineStr"/>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="3" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="4" t="inlineStr"/>
+      <c r="B79" s="4" t="inlineStr"/>
+      <c r="C79" s="5" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr"/>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr"/>
+      <c r="H79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="2" t="inlineStr"/>
+      <c r="B80" s="2" t="inlineStr"/>
+      <c r="C80" s="3" t="inlineStr"/>
+      <c r="D80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="4" t="inlineStr"/>
+      <c r="B81" s="4" t="inlineStr"/>
+      <c r="C81" s="5" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr"/>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr"/>
+      <c r="H81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="2" t="inlineStr"/>
+      <c r="B82" s="2" t="inlineStr"/>
+      <c r="C82" s="3" t="inlineStr"/>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="4" t="inlineStr"/>
+      <c r="B83" s="4" t="inlineStr"/>
+      <c r="C83" s="5" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr"/>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr"/>
+      <c r="H83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="2" t="inlineStr"/>
+      <c r="B84" s="2" t="inlineStr"/>
+      <c r="C84" s="3" t="inlineStr"/>
+      <c r="D84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="4" t="inlineStr"/>
+      <c r="B85" s="4" t="inlineStr"/>
+      <c r="C85" s="5" t="inlineStr"/>
+      <c r="D85" s="4" t="inlineStr"/>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr"/>
+      <c r="H85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="inlineStr"/>
+      <c r="B86" s="2" t="inlineStr"/>
+      <c r="C86" s="3" t="inlineStr"/>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="4" t="inlineStr"/>
+      <c r="B87" s="4" t="inlineStr"/>
+      <c r="C87" s="5" t="inlineStr"/>
+      <c r="D87" s="4" t="inlineStr"/>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr"/>
+      <c r="H87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="2" t="inlineStr"/>
+      <c r="B88" s="2" t="inlineStr"/>
+      <c r="C88" s="3" t="inlineStr"/>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="4" t="inlineStr"/>
+      <c r="B89" s="4" t="inlineStr"/>
+      <c r="C89" s="5" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr"/>
+      <c r="E89" s="4" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr"/>
+      <c r="G89" s="4" t="inlineStr"/>
+      <c r="H89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="inlineStr"/>
+      <c r="B90" s="2" t="inlineStr"/>
+      <c r="C90" s="3" t="inlineStr"/>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="4" t="inlineStr"/>
+      <c r="B91" s="4" t="inlineStr"/>
+      <c r="C91" s="5" t="inlineStr"/>
+      <c r="D91" s="4" t="inlineStr"/>
+      <c r="E91" s="4" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr"/>
+      <c r="H91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="2" t="inlineStr"/>
+      <c r="B92" s="2" t="inlineStr"/>
+      <c r="C92" s="3" t="inlineStr"/>
+      <c r="D92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="4" t="inlineStr"/>
+      <c r="B93" s="4" t="inlineStr"/>
+      <c r="C93" s="5" t="inlineStr"/>
+      <c r="D93" s="4" t="inlineStr"/>
+      <c r="E93" s="4" t="inlineStr"/>
+      <c r="F93" s="4" t="inlineStr"/>
+      <c r="G93" s="4" t="inlineStr"/>
+      <c r="H93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr"/>
+      <c r="B94" s="2" t="inlineStr"/>
+      <c r="C94" s="3" t="inlineStr"/>
+      <c r="D94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="4" t="inlineStr"/>
+      <c r="B95" s="4" t="inlineStr"/>
+      <c r="C95" s="5" t="inlineStr"/>
+      <c r="D95" s="4" t="inlineStr"/>
+      <c r="E95" s="4" t="inlineStr"/>
+      <c r="F95" s="4" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr"/>
+      <c r="H95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="inlineStr"/>
+      <c r="B96" s="2" t="inlineStr"/>
+      <c r="C96" s="3" t="inlineStr"/>
+      <c r="D96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="4" t="inlineStr"/>
+      <c r="B97" s="4" t="inlineStr"/>
+      <c r="C97" s="5" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr"/>
+      <c r="E97" s="4" t="inlineStr"/>
+      <c r="F97" s="4" t="inlineStr"/>
+      <c r="G97" s="4" t="inlineStr"/>
+      <c r="H97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="inlineStr"/>
+      <c r="B98" s="2" t="inlineStr"/>
+      <c r="C98" s="3" t="inlineStr"/>
+      <c r="D98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="4" t="inlineStr"/>
+      <c r="B99" s="4" t="inlineStr"/>
+      <c r="C99" s="5" t="inlineStr"/>
+      <c r="D99" s="4" t="inlineStr"/>
+      <c r="E99" s="4" t="inlineStr"/>
+      <c r="F99" s="4" t="inlineStr"/>
+      <c r="G99" s="4" t="inlineStr"/>
+      <c r="H99" s="4" t="inlineStr"/>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="2" t="inlineStr"/>
+      <c r="B100" s="2" t="inlineStr"/>
+      <c r="C100" s="3" t="inlineStr"/>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="4" t="inlineStr"/>
+      <c r="B101" s="4" t="inlineStr"/>
+      <c r="C101" s="5" t="inlineStr"/>
+      <c r="D101" s="4" t="inlineStr"/>
+      <c r="E101" s="4" t="inlineStr"/>
+      <c r="F101" s="4" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr"/>
+      <c r="H101" s="4" t="inlineStr"/>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="2" t="inlineStr"/>
+      <c r="B102" s="2" t="inlineStr"/>
+      <c r="C102" s="3" t="inlineStr"/>
+      <c r="D102" s="2" t="inlineStr"/>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="4" t="inlineStr"/>
+      <c r="B103" s="4" t="inlineStr"/>
+      <c r="C103" s="5" t="inlineStr"/>
+      <c r="D103" s="4" t="inlineStr"/>
+      <c r="E103" s="4" t="inlineStr"/>
+      <c r="F103" s="4" t="inlineStr"/>
+      <c r="G103" s="4" t="inlineStr"/>
+      <c r="H103" s="4" t="inlineStr"/>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="2" t="inlineStr"/>
+      <c r="B104" s="2" t="inlineStr"/>
+      <c r="C104" s="3" t="inlineStr"/>
+      <c r="D104" s="2" t="inlineStr"/>
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="4" t="inlineStr"/>
+      <c r="B105" s="4" t="inlineStr"/>
+      <c r="C105" s="5" t="inlineStr"/>
+      <c r="D105" s="4" t="inlineStr"/>
+      <c r="E105" s="4" t="inlineStr"/>
+      <c r="F105" s="4" t="inlineStr"/>
+      <c r="G105" s="4" t="inlineStr"/>
+      <c r="H105" s="4" t="inlineStr"/>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="2" t="inlineStr"/>
+      <c r="B106" s="2" t="inlineStr"/>
+      <c r="C106" s="3" t="inlineStr"/>
+      <c r="D106" s="2" t="inlineStr"/>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="4" t="inlineStr"/>
+      <c r="B107" s="4" t="inlineStr"/>
+      <c r="C107" s="5" t="inlineStr"/>
+      <c r="D107" s="4" t="inlineStr"/>
+      <c r="E107" s="4" t="inlineStr"/>
+      <c r="F107" s="4" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr"/>
+      <c r="H107" s="4" t="inlineStr"/>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="2" t="inlineStr"/>
+      <c r="B108" s="2" t="inlineStr"/>
+      <c r="C108" s="3" t="inlineStr"/>
+      <c r="D108" s="2" t="inlineStr"/>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="4" t="inlineStr"/>
+      <c r="B109" s="4" t="inlineStr"/>
+      <c r="C109" s="5" t="inlineStr"/>
+      <c r="D109" s="4" t="inlineStr"/>
+      <c r="E109" s="4" t="inlineStr"/>
+      <c r="F109" s="4" t="inlineStr"/>
+      <c r="G109" s="4" t="inlineStr"/>
+      <c r="H109" s="4" t="inlineStr"/>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="2" t="inlineStr"/>
+      <c r="B110" s="2" t="inlineStr"/>
+      <c r="C110" s="3" t="inlineStr"/>
+      <c r="D110" s="2" t="inlineStr"/>
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr"/>
+      <c r="H110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="4" t="inlineStr"/>
+      <c r="B111" s="4" t="inlineStr"/>
+      <c r="C111" s="5" t="inlineStr"/>
+      <c r="D111" s="4" t="inlineStr"/>
+      <c r="E111" s="4" t="inlineStr"/>
+      <c r="F111" s="4" t="inlineStr"/>
+      <c r="G111" s="4" t="inlineStr"/>
+      <c r="H111" s="4" t="inlineStr"/>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="2" t="inlineStr"/>
+      <c r="B112" s="2" t="inlineStr"/>
+      <c r="C112" s="3" t="inlineStr"/>
+      <c r="D112" s="2" t="inlineStr"/>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr"/>
+      <c r="G112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="4" t="inlineStr"/>
+      <c r="B113" s="4" t="inlineStr"/>
+      <c r="C113" s="5" t="inlineStr"/>
+      <c r="D113" s="4" t="inlineStr"/>
+      <c r="E113" s="4" t="inlineStr"/>
+      <c r="F113" s="4" t="inlineStr"/>
+      <c r="G113" s="4" t="inlineStr"/>
+      <c r="H113" s="4" t="inlineStr"/>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="2" t="inlineStr"/>
+      <c r="B114" s="2" t="inlineStr"/>
+      <c r="C114" s="3" t="inlineStr"/>
+      <c r="D114" s="2" t="inlineStr"/>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr"/>
+      <c r="H114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="4" t="inlineStr"/>
+      <c r="B115" s="4" t="inlineStr"/>
+      <c r="C115" s="5" t="inlineStr"/>
+      <c r="D115" s="4" t="inlineStr"/>
+      <c r="E115" s="4" t="inlineStr"/>
+      <c r="F115" s="4" t="inlineStr"/>
+      <c r="G115" s="4" t="inlineStr"/>
+      <c r="H115" s="4" t="inlineStr"/>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="2" t="inlineStr"/>
+      <c r="B116" s="2" t="inlineStr"/>
+      <c r="C116" s="3" t="inlineStr"/>
+      <c r="D116" s="2" t="inlineStr"/>
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="4" t="inlineStr"/>
+      <c r="B117" s="4" t="inlineStr"/>
+      <c r="C117" s="5" t="inlineStr"/>
+      <c r="D117" s="4" t="inlineStr"/>
+      <c r="E117" s="4" t="inlineStr"/>
+      <c r="F117" s="4" t="inlineStr"/>
+      <c r="G117" s="4" t="inlineStr"/>
+      <c r="H117" s="4" t="inlineStr"/>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="2" t="inlineStr"/>
+      <c r="B118" s="2" t="inlineStr"/>
+      <c r="C118" s="3" t="inlineStr"/>
+      <c r="D118" s="2" t="inlineStr"/>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr"/>
+      <c r="H118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="4" t="inlineStr"/>
+      <c r="B119" s="4" t="inlineStr"/>
+      <c r="C119" s="5" t="inlineStr"/>
+      <c r="D119" s="4" t="inlineStr"/>
+      <c r="E119" s="4" t="inlineStr"/>
+      <c r="F119" s="4" t="inlineStr"/>
+      <c r="G119" s="4" t="inlineStr"/>
+      <c r="H119" s="4" t="inlineStr"/>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="2" t="inlineStr"/>
+      <c r="B120" s="2" t="inlineStr"/>
+      <c r="C120" s="3" t="inlineStr"/>
+      <c r="D120" s="2" t="inlineStr"/>
+      <c r="E120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="4" t="inlineStr"/>
+      <c r="B121" s="4" t="inlineStr"/>
+      <c r="C121" s="5" t="inlineStr"/>
+      <c r="D121" s="4" t="inlineStr"/>
+      <c r="E121" s="4" t="inlineStr"/>
+      <c r="F121" s="4" t="inlineStr"/>
+      <c r="G121" s="4" t="inlineStr"/>
+      <c r="H121" s="4" t="inlineStr"/>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="2" t="inlineStr"/>
+      <c r="B122" s="2" t="inlineStr"/>
+      <c r="C122" s="3" t="inlineStr"/>
+      <c r="D122" s="2" t="inlineStr"/>
+      <c r="E122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="inlineStr"/>
+      <c r="G122" s="2" t="inlineStr"/>
+      <c r="H122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="4" t="inlineStr"/>
+      <c r="B123" s="4" t="inlineStr"/>
+      <c r="C123" s="5" t="inlineStr"/>
+      <c r="D123" s="4" t="inlineStr"/>
+      <c r="E123" s="4" t="inlineStr"/>
+      <c r="F123" s="4" t="inlineStr"/>
+      <c r="G123" s="4" t="inlineStr"/>
+      <c r="H123" s="4" t="inlineStr"/>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="2" t="inlineStr"/>
+      <c r="B124" s="2" t="inlineStr"/>
+      <c r="C124" s="3" t="inlineStr"/>
+      <c r="D124" s="2" t="inlineStr"/>
+      <c r="E124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="inlineStr"/>
+      <c r="G124" s="2" t="inlineStr"/>
+      <c r="H124" s="2" t="inlineStr"/>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="4" t="inlineStr"/>
+      <c r="B125" s="4" t="inlineStr"/>
+      <c r="C125" s="5" t="inlineStr"/>
+      <c r="D125" s="4" t="inlineStr"/>
+      <c r="E125" s="4" t="inlineStr"/>
+      <c r="F125" s="4" t="inlineStr"/>
+      <c r="G125" s="4" t="inlineStr"/>
+      <c r="H125" s="4" t="inlineStr"/>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="2" t="inlineStr"/>
+      <c r="B126" s="2" t="inlineStr"/>
+      <c r="C126" s="3" t="inlineStr"/>
+      <c r="D126" s="2" t="inlineStr"/>
+      <c r="E126" s="2" t="inlineStr"/>
+      <c r="F126" s="2" t="inlineStr"/>
+      <c r="G126" s="2" t="inlineStr"/>
+      <c r="H126" s="2" t="inlineStr"/>
+    </row>
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="4" t="inlineStr"/>
+      <c r="B127" s="4" t="inlineStr"/>
+      <c r="C127" s="5" t="inlineStr"/>
+      <c r="D127" s="4" t="inlineStr"/>
+      <c r="E127" s="4" t="inlineStr"/>
+      <c r="F127" s="4" t="inlineStr"/>
+      <c r="G127" s="4" t="inlineStr"/>
+      <c r="H127" s="4" t="inlineStr"/>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="2" t="inlineStr"/>
+      <c r="B128" s="2" t="inlineStr"/>
+      <c r="C128" s="3" t="inlineStr"/>
+      <c r="D128" s="2" t="inlineStr"/>
+      <c r="E128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="inlineStr"/>
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="4" t="inlineStr"/>
+      <c r="B129" s="4" t="inlineStr"/>
+      <c r="C129" s="5" t="inlineStr"/>
+      <c r="D129" s="4" t="inlineStr"/>
+      <c r="E129" s="4" t="inlineStr"/>
+      <c r="F129" s="4" t="inlineStr"/>
+      <c r="G129" s="4" t="inlineStr"/>
+      <c r="H129" s="4" t="inlineStr"/>
+    </row>
+    <row r="130" ht="22" customHeight="1">
+      <c r="A130" s="2" t="inlineStr"/>
+      <c r="B130" s="2" t="inlineStr"/>
+      <c r="C130" s="3" t="inlineStr"/>
+      <c r="D130" s="2" t="inlineStr"/>
+      <c r="E130" s="2" t="inlineStr"/>
+      <c r="F130" s="2" t="inlineStr"/>
+      <c r="G130" s="2" t="inlineStr"/>
+      <c r="H130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131" ht="22" customHeight="1">
+      <c r="A131" s="4" t="inlineStr"/>
+      <c r="B131" s="4" t="inlineStr"/>
+      <c r="C131" s="5" t="inlineStr"/>
+      <c r="D131" s="4" t="inlineStr"/>
+      <c r="E131" s="4" t="inlineStr"/>
+      <c r="F131" s="4" t="inlineStr"/>
+      <c r="G131" s="4" t="inlineStr"/>
+      <c r="H131" s="4" t="inlineStr"/>
+    </row>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="2" t="inlineStr"/>
+      <c r="B132" s="2" t="inlineStr"/>
+      <c r="C132" s="3" t="inlineStr"/>
+      <c r="D132" s="2" t="inlineStr"/>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr"/>
+      <c r="G132" s="2" t="inlineStr"/>
+      <c r="H132" s="2" t="inlineStr"/>
+    </row>
+    <row r="133" ht="22" customHeight="1">
+      <c r="A133" s="4" t="inlineStr"/>
+      <c r="B133" s="4" t="inlineStr"/>
+      <c r="C133" s="5" t="inlineStr"/>
+      <c r="D133" s="4" t="inlineStr"/>
+      <c r="E133" s="4" t="inlineStr"/>
+      <c r="F133" s="4" t="inlineStr"/>
+      <c r="G133" s="4" t="inlineStr"/>
+      <c r="H133" s="4" t="inlineStr"/>
+    </row>
+    <row r="134" ht="22" customHeight="1">
+      <c r="A134" s="2" t="inlineStr"/>
+      <c r="B134" s="2" t="inlineStr"/>
+      <c r="C134" s="3" t="inlineStr"/>
+      <c r="D134" s="2" t="inlineStr"/>
+      <c r="E134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr"/>
+      <c r="G134" s="2" t="inlineStr"/>
+      <c r="H134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="4" t="inlineStr"/>
+      <c r="B135" s="4" t="inlineStr"/>
+      <c r="C135" s="5" t="inlineStr"/>
+      <c r="D135" s="4" t="inlineStr"/>
+      <c r="E135" s="4" t="inlineStr"/>
+      <c r="F135" s="4" t="inlineStr"/>
+      <c r="G135" s="4" t="inlineStr"/>
+      <c r="H135" s="4" t="inlineStr"/>
+    </row>
+    <row r="136" ht="22" customHeight="1">
+      <c r="A136" s="2" t="inlineStr"/>
+      <c r="B136" s="2" t="inlineStr"/>
+      <c r="C136" s="3" t="inlineStr"/>
+      <c r="D136" s="2" t="inlineStr"/>
+      <c r="E136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="inlineStr"/>
+      <c r="G136" s="2" t="inlineStr"/>
+      <c r="H136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137" ht="22" customHeight="1">
+      <c r="A137" s="4" t="inlineStr"/>
+      <c r="B137" s="4" t="inlineStr"/>
+      <c r="C137" s="5" t="inlineStr"/>
+      <c r="D137" s="4" t="inlineStr"/>
+      <c r="E137" s="4" t="inlineStr"/>
+      <c r="F137" s="4" t="inlineStr"/>
+      <c r="G137" s="4" t="inlineStr"/>
+      <c r="H137" s="4" t="inlineStr"/>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="2" t="inlineStr"/>
+      <c r="B138" s="2" t="inlineStr"/>
+      <c r="C138" s="3" t="inlineStr"/>
+      <c r="D138" s="2" t="inlineStr"/>
+      <c r="E138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr"/>
+      <c r="G138" s="2" t="inlineStr"/>
+      <c r="H138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139" ht="22" customHeight="1">
+      <c r="A139" s="4" t="inlineStr"/>
+      <c r="B139" s="4" t="inlineStr"/>
+      <c r="C139" s="5" t="inlineStr"/>
+      <c r="D139" s="4" t="inlineStr"/>
+      <c r="E139" s="4" t="inlineStr"/>
+      <c r="F139" s="4" t="inlineStr"/>
+      <c r="G139" s="4" t="inlineStr"/>
+      <c r="H139" s="4" t="inlineStr"/>
+    </row>
+    <row r="140" ht="22" customHeight="1">
+      <c r="A140" s="2" t="inlineStr"/>
+      <c r="B140" s="2" t="inlineStr"/>
+      <c r="C140" s="3" t="inlineStr"/>
+      <c r="D140" s="2" t="inlineStr"/>
+      <c r="E140" s="2" t="inlineStr"/>
+      <c r="F140" s="2" t="inlineStr"/>
+      <c r="G140" s="2" t="inlineStr"/>
+      <c r="H140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="4" t="inlineStr"/>
+      <c r="B141" s="4" t="inlineStr"/>
+      <c r="C141" s="5" t="inlineStr"/>
+      <c r="D141" s="4" t="inlineStr"/>
+      <c r="E141" s="4" t="inlineStr"/>
+      <c r="F141" s="4" t="inlineStr"/>
+      <c r="G141" s="4" t="inlineStr"/>
+      <c r="H141" s="4" t="inlineStr"/>
+    </row>
+    <row r="142" ht="22" customHeight="1">
+      <c r="A142" s="2" t="inlineStr"/>
+      <c r="B142" s="2" t="inlineStr"/>
+      <c r="C142" s="3" t="inlineStr"/>
+      <c r="D142" s="2" t="inlineStr"/>
+      <c r="E142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr"/>
+      <c r="G142" s="2" t="inlineStr"/>
+      <c r="H142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143" ht="22" customHeight="1">
+      <c r="A143" s="4" t="inlineStr"/>
+      <c r="B143" s="4" t="inlineStr"/>
+      <c r="C143" s="5" t="inlineStr"/>
+      <c r="D143" s="4" t="inlineStr"/>
+      <c r="E143" s="4" t="inlineStr"/>
+      <c r="F143" s="4" t="inlineStr"/>
+      <c r="G143" s="4" t="inlineStr"/>
+      <c r="H143" s="4" t="inlineStr"/>
+    </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="2" t="inlineStr"/>
+      <c r="B144" s="2" t="inlineStr"/>
+      <c r="C144" s="3" t="inlineStr"/>
+      <c r="D144" s="2" t="inlineStr"/>
+      <c r="E144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr"/>
+      <c r="G144" s="2" t="inlineStr"/>
+      <c r="H144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="4" t="inlineStr"/>
+      <c r="B145" s="4" t="inlineStr"/>
+      <c r="C145" s="5" t="inlineStr"/>
+      <c r="D145" s="4" t="inlineStr"/>
+      <c r="E145" s="4" t="inlineStr"/>
+      <c r="F145" s="4" t="inlineStr"/>
+      <c r="G145" s="4" t="inlineStr"/>
+      <c r="H145" s="4" t="inlineStr"/>
+    </row>
+    <row r="146" ht="22" customHeight="1">
+      <c r="A146" s="2" t="inlineStr"/>
+      <c r="B146" s="2" t="inlineStr"/>
+      <c r="C146" s="3" t="inlineStr"/>
+      <c r="D146" s="2" t="inlineStr"/>
+      <c r="E146" s="2" t="inlineStr"/>
+      <c r="F146" s="2" t="inlineStr"/>
+      <c r="G146" s="2" t="inlineStr"/>
+      <c r="H146" s="2" t="inlineStr"/>
+    </row>
+    <row r="147" ht="22" customHeight="1">
+      <c r="A147" s="4" t="inlineStr"/>
+      <c r="B147" s="4" t="inlineStr"/>
+      <c r="C147" s="5" t="inlineStr"/>
+      <c r="D147" s="4" t="inlineStr"/>
+      <c r="E147" s="4" t="inlineStr"/>
+      <c r="F147" s="4" t="inlineStr"/>
+      <c r="G147" s="4" t="inlineStr"/>
+      <c r="H147" s="4" t="inlineStr"/>
+    </row>
+    <row r="148" ht="22" customHeight="1">
+      <c r="A148" s="2" t="inlineStr"/>
+      <c r="B148" s="2" t="inlineStr"/>
+      <c r="C148" s="3" t="inlineStr"/>
+      <c r="D148" s="2" t="inlineStr"/>
+      <c r="E148" s="2" t="inlineStr"/>
+      <c r="F148" s="2" t="inlineStr"/>
+      <c r="G148" s="2" t="inlineStr"/>
+      <c r="H148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149" ht="22" customHeight="1">
+      <c r="A149" s="4" t="inlineStr"/>
+      <c r="B149" s="4" t="inlineStr"/>
+      <c r="C149" s="5" t="inlineStr"/>
+      <c r="D149" s="4" t="inlineStr"/>
+      <c r="E149" s="4" t="inlineStr"/>
+      <c r="F149" s="4" t="inlineStr"/>
+      <c r="G149" s="4" t="inlineStr"/>
+      <c r="H149" s="4" t="inlineStr"/>
+    </row>
+    <row r="150" ht="22" customHeight="1">
+      <c r="A150" s="2" t="inlineStr"/>
+      <c r="B150" s="2" t="inlineStr"/>
+      <c r="C150" s="3" t="inlineStr"/>
+      <c r="D150" s="2" t="inlineStr"/>
+      <c r="E150" s="2" t="inlineStr"/>
+      <c r="F150" s="2" t="inlineStr"/>
+      <c r="G150" s="2" t="inlineStr"/>
+      <c r="H150" s="2" t="inlineStr"/>
+    </row>
+    <row r="151" ht="22" customHeight="1">
+      <c r="A151" s="4" t="inlineStr"/>
+      <c r="B151" s="4" t="inlineStr"/>
+      <c r="C151" s="5" t="inlineStr"/>
+      <c r="D151" s="4" t="inlineStr"/>
+      <c r="E151" s="4" t="inlineStr"/>
+      <c r="F151" s="4" t="inlineStr"/>
+      <c r="G151" s="4" t="inlineStr"/>
+      <c r="H151" s="4" t="inlineStr"/>
+    </row>
+    <row r="152" ht="22" customHeight="1">
+      <c r="A152" s="2" t="inlineStr"/>
+      <c r="B152" s="2" t="inlineStr"/>
+      <c r="C152" s="3" t="inlineStr"/>
+      <c r="D152" s="2" t="inlineStr"/>
+      <c r="E152" s="2" t="inlineStr"/>
+      <c r="F152" s="2" t="inlineStr"/>
+      <c r="G152" s="2" t="inlineStr"/>
+      <c r="H152" s="2" t="inlineStr"/>
+    </row>
+    <row r="153" ht="22" customHeight="1">
+      <c r="A153" s="4" t="inlineStr"/>
+      <c r="B153" s="4" t="inlineStr"/>
+      <c r="C153" s="5" t="inlineStr"/>
+      <c r="D153" s="4" t="inlineStr"/>
+      <c r="E153" s="4" t="inlineStr"/>
+      <c r="F153" s="4" t="inlineStr"/>
+      <c r="G153" s="4" t="inlineStr"/>
+      <c r="H153" s="4" t="inlineStr"/>
+    </row>
+    <row r="154" ht="22" customHeight="1">
+      <c r="A154" s="2" t="inlineStr"/>
+      <c r="B154" s="2" t="inlineStr"/>
+      <c r="C154" s="3" t="inlineStr"/>
+      <c r="D154" s="2" t="inlineStr"/>
+      <c r="E154" s="2" t="inlineStr"/>
+      <c r="F154" s="2" t="inlineStr"/>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155" ht="22" customHeight="1">
+      <c r="A155" s="4" t="inlineStr"/>
+      <c r="B155" s="4" t="inlineStr"/>
+      <c r="C155" s="5" t="inlineStr"/>
+      <c r="D155" s="4" t="inlineStr"/>
+      <c r="E155" s="4" t="inlineStr"/>
+      <c r="F155" s="4" t="inlineStr"/>
+      <c r="G155" s="4" t="inlineStr"/>
+      <c r="H155" s="4" t="inlineStr"/>
+    </row>
+    <row r="156" ht="22" customHeight="1">
+      <c r="A156" s="2" t="inlineStr"/>
+      <c r="B156" s="2" t="inlineStr"/>
+      <c r="C156" s="3" t="inlineStr"/>
+      <c r="D156" s="2" t="inlineStr"/>
+      <c r="E156" s="2" t="inlineStr"/>
+      <c r="F156" s="2" t="inlineStr"/>
+      <c r="G156" s="2" t="inlineStr"/>
+      <c r="H156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157" ht="22" customHeight="1">
+      <c r="A157" s="4" t="inlineStr"/>
+      <c r="B157" s="4" t="inlineStr"/>
+      <c r="C157" s="5" t="inlineStr"/>
+      <c r="D157" s="4" t="inlineStr"/>
+      <c r="E157" s="4" t="inlineStr"/>
+      <c r="F157" s="4" t="inlineStr"/>
+      <c r="G157" s="4" t="inlineStr"/>
+      <c r="H157" s="4" t="inlineStr"/>
+    </row>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="2" t="inlineStr"/>
+      <c r="B158" s="2" t="inlineStr"/>
+      <c r="C158" s="3" t="inlineStr"/>
+      <c r="D158" s="2" t="inlineStr"/>
+      <c r="E158" s="2" t="inlineStr"/>
+      <c r="F158" s="2" t="inlineStr"/>
+      <c r="G158" s="2" t="inlineStr"/>
+      <c r="H158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159" ht="22" customHeight="1">
+      <c r="A159" s="4" t="inlineStr"/>
+      <c r="B159" s="4" t="inlineStr"/>
+      <c r="C159" s="5" t="inlineStr"/>
+      <c r="D159" s="4" t="inlineStr"/>
+      <c r="E159" s="4" t="inlineStr"/>
+      <c r="F159" s="4" t="inlineStr"/>
+      <c r="G159" s="4" t="inlineStr"/>
+      <c r="H159" s="4" t="inlineStr"/>
+    </row>
+    <row r="160" ht="22" customHeight="1">
+      <c r="A160" s="2" t="inlineStr"/>
+      <c r="B160" s="2" t="inlineStr"/>
+      <c r="C160" s="3" t="inlineStr"/>
+      <c r="D160" s="2" t="inlineStr"/>
+      <c r="E160" s="2" t="inlineStr"/>
+      <c r="F160" s="2" t="inlineStr"/>
+      <c r="G160" s="2" t="inlineStr"/>
+      <c r="H160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161" ht="22" customHeight="1">
+      <c r="A161" s="4" t="inlineStr"/>
+      <c r="B161" s="4" t="inlineStr"/>
+      <c r="C161" s="5" t="inlineStr"/>
+      <c r="D161" s="4" t="inlineStr"/>
+      <c r="E161" s="4" t="inlineStr"/>
+      <c r="F161" s="4" t="inlineStr"/>
+      <c r="G161" s="4" t="inlineStr"/>
+      <c r="H161" s="4" t="inlineStr"/>
+    </row>
+    <row r="162" ht="22" customHeight="1">
+      <c r="A162" s="2" t="inlineStr"/>
+      <c r="B162" s="2" t="inlineStr"/>
+      <c r="C162" s="3" t="inlineStr"/>
+      <c r="D162" s="2" t="inlineStr"/>
+      <c r="E162" s="2" t="inlineStr"/>
+      <c r="F162" s="2" t="inlineStr"/>
+      <c r="G162" s="2" t="inlineStr"/>
+      <c r="H162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163" ht="22" customHeight="1">
+      <c r="A163" s="4" t="inlineStr"/>
+      <c r="B163" s="4" t="inlineStr"/>
+      <c r="C163" s="5" t="inlineStr"/>
+      <c r="D163" s="4" t="inlineStr"/>
+      <c r="E163" s="4" t="inlineStr"/>
+      <c r="F163" s="4" t="inlineStr"/>
+      <c r="G163" s="4" t="inlineStr"/>
+      <c r="H163" s="4" t="inlineStr"/>
+    </row>
+    <row r="164" ht="22" customHeight="1">
+      <c r="A164" s="2" t="inlineStr"/>
+      <c r="B164" s="2" t="inlineStr"/>
+      <c r="C164" s="3" t="inlineStr"/>
+      <c r="D164" s="2" t="inlineStr"/>
+      <c r="E164" s="2" t="inlineStr"/>
+      <c r="F164" s="2" t="inlineStr"/>
+      <c r="G164" s="2" t="inlineStr"/>
+      <c r="H164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165" ht="22" customHeight="1">
+      <c r="A165" s="4" t="inlineStr"/>
+      <c r="B165" s="4" t="inlineStr"/>
+      <c r="C165" s="5" t="inlineStr"/>
+      <c r="D165" s="4" t="inlineStr"/>
+      <c r="E165" s="4" t="inlineStr"/>
+      <c r="F165" s="4" t="inlineStr"/>
+      <c r="G165" s="4" t="inlineStr"/>
+      <c r="H165" s="4" t="inlineStr"/>
+    </row>
+    <row r="166" ht="22" customHeight="1">
+      <c r="A166" s="2" t="inlineStr"/>
+      <c r="B166" s="2" t="inlineStr"/>
+      <c r="C166" s="3" t="inlineStr"/>
+      <c r="D166" s="2" t="inlineStr"/>
+      <c r="E166" s="2" t="inlineStr"/>
+      <c r="F166" s="2" t="inlineStr"/>
+      <c r="G166" s="2" t="inlineStr"/>
+      <c r="H166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167" ht="22" customHeight="1">
+      <c r="A167" s="4" t="inlineStr"/>
+      <c r="B167" s="4" t="inlineStr"/>
+      <c r="C167" s="5" t="inlineStr"/>
+      <c r="D167" s="4" t="inlineStr"/>
+      <c r="E167" s="4" t="inlineStr"/>
+      <c r="F167" s="4" t="inlineStr"/>
+      <c r="G167" s="4" t="inlineStr"/>
+      <c r="H167" s="4" t="inlineStr"/>
+    </row>
+    <row r="168" ht="22" customHeight="1">
+      <c r="A168" s="2" t="inlineStr"/>
+      <c r="B168" s="2" t="inlineStr"/>
+      <c r="C168" s="3" t="inlineStr"/>
+      <c r="D168" s="2" t="inlineStr"/>
+      <c r="E168" s="2" t="inlineStr"/>
+      <c r="F168" s="2" t="inlineStr"/>
+      <c r="G168" s="2" t="inlineStr"/>
+      <c r="H168" s="2" t="inlineStr"/>
+    </row>
+    <row r="169" ht="22" customHeight="1">
+      <c r="A169" s="4" t="inlineStr"/>
+      <c r="B169" s="4" t="inlineStr"/>
+      <c r="C169" s="5" t="inlineStr"/>
+      <c r="D169" s="4" t="inlineStr"/>
+      <c r="E169" s="4" t="inlineStr"/>
+      <c r="F169" s="4" t="inlineStr"/>
+      <c r="G169" s="4" t="inlineStr"/>
+      <c r="H169" s="4" t="inlineStr"/>
+    </row>
+    <row r="170" ht="22" customHeight="1">
+      <c r="A170" s="2" t="inlineStr"/>
+      <c r="B170" s="2" t="inlineStr"/>
+      <c r="C170" s="3" t="inlineStr"/>
+      <c r="D170" s="2" t="inlineStr"/>
+      <c r="E170" s="2" t="inlineStr"/>
+      <c r="F170" s="2" t="inlineStr"/>
+      <c r="G170" s="2" t="inlineStr"/>
+      <c r="H170" s="2" t="inlineStr"/>
+    </row>
+    <row r="171" ht="22" customHeight="1">
+      <c r="A171" s="4" t="inlineStr"/>
+      <c r="B171" s="4" t="inlineStr"/>
+      <c r="C171" s="5" t="inlineStr"/>
+      <c r="D171" s="4" t="inlineStr"/>
+      <c r="E171" s="4" t="inlineStr"/>
+      <c r="F171" s="4" t="inlineStr"/>
+      <c r="G171" s="4" t="inlineStr"/>
+      <c r="H171" s="4" t="inlineStr"/>
+    </row>
+    <row r="172" ht="22" customHeight="1">
+      <c r="A172" s="2" t="inlineStr"/>
+      <c r="B172" s="2" t="inlineStr"/>
+      <c r="C172" s="3" t="inlineStr"/>
+      <c r="D172" s="2" t="inlineStr"/>
+      <c r="E172" s="2" t="inlineStr"/>
+      <c r="F172" s="2" t="inlineStr"/>
+      <c r="G172" s="2" t="inlineStr"/>
+      <c r="H172" s="2" t="inlineStr"/>
+    </row>
+    <row r="173" ht="22" customHeight="1">
+      <c r="A173" s="4" t="inlineStr"/>
+      <c r="B173" s="4" t="inlineStr"/>
+      <c r="C173" s="5" t="inlineStr"/>
+      <c r="D173" s="4" t="inlineStr"/>
+      <c r="E173" s="4" t="inlineStr"/>
+      <c r="F173" s="4" t="inlineStr"/>
+      <c r="G173" s="4" t="inlineStr"/>
+      <c r="H173" s="4" t="inlineStr"/>
+    </row>
+    <row r="174" ht="22" customHeight="1">
+      <c r="A174" s="2" t="inlineStr"/>
+      <c r="B174" s="2" t="inlineStr"/>
+      <c r="C174" s="3" t="inlineStr"/>
+      <c r="D174" s="2" t="inlineStr"/>
+      <c r="E174" s="2" t="inlineStr"/>
+      <c r="F174" s="2" t="inlineStr"/>
+      <c r="G174" s="2" t="inlineStr"/>
+      <c r="H174" s="2" t="inlineStr"/>
+    </row>
+    <row r="175" ht="22" customHeight="1">
+      <c r="A175" s="4" t="inlineStr"/>
+      <c r="B175" s="4" t="inlineStr"/>
+      <c r="C175" s="5" t="inlineStr"/>
+      <c r="D175" s="4" t="inlineStr"/>
+      <c r="E175" s="4" t="inlineStr"/>
+      <c r="F175" s="4" t="inlineStr"/>
+      <c r="G175" s="4" t="inlineStr"/>
+      <c r="H175" s="4" t="inlineStr"/>
+    </row>
+    <row r="176" ht="22" customHeight="1">
+      <c r="A176" s="2" t="inlineStr"/>
+      <c r="B176" s="2" t="inlineStr"/>
+      <c r="C176" s="3" t="inlineStr"/>
+      <c r="D176" s="2" t="inlineStr"/>
+      <c r="E176" s="2" t="inlineStr"/>
+      <c r="F176" s="2" t="inlineStr"/>
+      <c r="G176" s="2" t="inlineStr"/>
+      <c r="H176" s="2" t="inlineStr"/>
+    </row>
+    <row r="177" ht="22" customHeight="1">
+      <c r="A177" s="4" t="inlineStr"/>
+      <c r="B177" s="4" t="inlineStr"/>
+      <c r="C177" s="5" t="inlineStr"/>
+      <c r="D177" s="4" t="inlineStr"/>
+      <c r="E177" s="4" t="inlineStr"/>
+      <c r="F177" s="4" t="inlineStr"/>
+      <c r="G177" s="4" t="inlineStr"/>
+      <c r="H177" s="4" t="inlineStr"/>
+    </row>
+    <row r="178" ht="22" customHeight="1">
+      <c r="A178" s="2" t="inlineStr"/>
+      <c r="B178" s="2" t="inlineStr"/>
+      <c r="C178" s="3" t="inlineStr"/>
+      <c r="D178" s="2" t="inlineStr"/>
+      <c r="E178" s="2" t="inlineStr"/>
+      <c r="F178" s="2" t="inlineStr"/>
+      <c r="G178" s="2" t="inlineStr"/>
+      <c r="H178" s="2" t="inlineStr"/>
+    </row>
+    <row r="179" ht="22" customHeight="1">
+      <c r="A179" s="4" t="inlineStr"/>
+      <c r="B179" s="4" t="inlineStr"/>
+      <c r="C179" s="5" t="inlineStr"/>
+      <c r="D179" s="4" t="inlineStr"/>
+      <c r="E179" s="4" t="inlineStr"/>
+      <c r="F179" s="4" t="inlineStr"/>
+      <c r="G179" s="4" t="inlineStr"/>
+      <c r="H179" s="4" t="inlineStr"/>
+    </row>
+    <row r="180" ht="22" customHeight="1">
+      <c r="A180" s="2" t="inlineStr"/>
+      <c r="B180" s="2" t="inlineStr"/>
+      <c r="C180" s="3" t="inlineStr"/>
+      <c r="D180" s="2" t="inlineStr"/>
+      <c r="E180" s="2" t="inlineStr"/>
+      <c r="F180" s="2" t="inlineStr"/>
+      <c r="G180" s="2" t="inlineStr"/>
+      <c r="H180" s="2" t="inlineStr"/>
+    </row>
+    <row r="181" ht="22" customHeight="1">
+      <c r="A181" s="4" t="inlineStr"/>
+      <c r="B181" s="4" t="inlineStr"/>
+      <c r="C181" s="5" t="inlineStr"/>
+      <c r="D181" s="4" t="inlineStr"/>
+      <c r="E181" s="4" t="inlineStr"/>
+      <c r="F181" s="4" t="inlineStr"/>
+      <c r="G181" s="4" t="inlineStr"/>
+      <c r="H181" s="4" t="inlineStr"/>
+    </row>
+    <row r="182" ht="22" customHeight="1">
+      <c r="A182" s="2" t="inlineStr"/>
+      <c r="B182" s="2" t="inlineStr"/>
+      <c r="C182" s="3" t="inlineStr"/>
+      <c r="D182" s="2" t="inlineStr"/>
+      <c r="E182" s="2" t="inlineStr"/>
+      <c r="F182" s="2" t="inlineStr"/>
+      <c r="G182" s="2" t="inlineStr"/>
+      <c r="H182" s="2" t="inlineStr"/>
+    </row>
+    <row r="183" ht="22" customHeight="1">
+      <c r="A183" s="4" t="inlineStr"/>
+      <c r="B183" s="4" t="inlineStr"/>
+      <c r="C183" s="5" t="inlineStr"/>
+      <c r="D183" s="4" t="inlineStr"/>
+      <c r="E183" s="4" t="inlineStr"/>
+      <c r="F183" s="4" t="inlineStr"/>
+      <c r="G183" s="4" t="inlineStr"/>
+      <c r="H183" s="4" t="inlineStr"/>
+    </row>
+    <row r="184" ht="22" customHeight="1">
+      <c r="A184" s="2" t="inlineStr"/>
+      <c r="B184" s="2" t="inlineStr"/>
+      <c r="C184" s="3" t="inlineStr"/>
+      <c r="D184" s="2" t="inlineStr"/>
+      <c r="E184" s="2" t="inlineStr"/>
+      <c r="F184" s="2" t="inlineStr"/>
+      <c r="G184" s="2" t="inlineStr"/>
+      <c r="H184" s="2" t="inlineStr"/>
+    </row>
+    <row r="185" ht="22" customHeight="1">
+      <c r="A185" s="4" t="inlineStr"/>
+      <c r="B185" s="4" t="inlineStr"/>
+      <c r="C185" s="5" t="inlineStr"/>
+      <c r="D185" s="4" t="inlineStr"/>
+      <c r="E185" s="4" t="inlineStr"/>
+      <c r="F185" s="4" t="inlineStr"/>
+      <c r="G185" s="4" t="inlineStr"/>
+      <c r="H185" s="4" t="inlineStr"/>
+    </row>
+    <row r="186" ht="22" customHeight="1">
+      <c r="A186" s="2" t="inlineStr"/>
+      <c r="B186" s="2" t="inlineStr"/>
+      <c r="C186" s="3" t="inlineStr"/>
+      <c r="D186" s="2" t="inlineStr"/>
+      <c r="E186" s="2" t="inlineStr"/>
+      <c r="F186" s="2" t="inlineStr"/>
+      <c r="G186" s="2" t="inlineStr"/>
+      <c r="H186" s="2" t="inlineStr"/>
+    </row>
+    <row r="187" ht="22" customHeight="1">
+      <c r="A187" s="4" t="inlineStr"/>
+      <c r="B187" s="4" t="inlineStr"/>
+      <c r="C187" s="5" t="inlineStr"/>
+      <c r="D187" s="4" t="inlineStr"/>
+      <c r="E187" s="4" t="inlineStr"/>
+      <c r="F187" s="4" t="inlineStr"/>
+      <c r="G187" s="4" t="inlineStr"/>
+      <c r="H187" s="4" t="inlineStr"/>
+    </row>
+    <row r="188" ht="22" customHeight="1">
+      <c r="A188" s="2" t="inlineStr"/>
+      <c r="B188" s="2" t="inlineStr"/>
+      <c r="C188" s="3" t="inlineStr"/>
+      <c r="D188" s="2" t="inlineStr"/>
+      <c r="E188" s="2" t="inlineStr"/>
+      <c r="F188" s="2" t="inlineStr"/>
+      <c r="G188" s="2" t="inlineStr"/>
+      <c r="H188" s="2" t="inlineStr"/>
+    </row>
+    <row r="189" ht="22" customHeight="1">
+      <c r="A189" s="4" t="inlineStr"/>
+      <c r="B189" s="4" t="inlineStr"/>
+      <c r="C189" s="5" t="inlineStr"/>
+      <c r="D189" s="4" t="inlineStr"/>
+      <c r="E189" s="4" t="inlineStr"/>
+      <c r="F189" s="4" t="inlineStr"/>
+      <c r="G189" s="4" t="inlineStr"/>
+      <c r="H189" s="4" t="inlineStr"/>
+    </row>
+    <row r="190" ht="22" customHeight="1">
+      <c r="A190" s="2" t="inlineStr"/>
+      <c r="B190" s="2" t="inlineStr"/>
+      <c r="C190" s="3" t="inlineStr"/>
+      <c r="D190" s="2" t="inlineStr"/>
+      <c r="E190" s="2" t="inlineStr"/>
+      <c r="F190" s="2" t="inlineStr"/>
+      <c r="G190" s="2" t="inlineStr"/>
+      <c r="H190" s="2" t="inlineStr"/>
+    </row>
+    <row r="191" ht="22" customHeight="1">
+      <c r="A191" s="4" t="inlineStr"/>
+      <c r="B191" s="4" t="inlineStr"/>
+      <c r="C191" s="5" t="inlineStr"/>
+      <c r="D191" s="4" t="inlineStr"/>
+      <c r="E191" s="4" t="inlineStr"/>
+      <c r="F191" s="4" t="inlineStr"/>
+      <c r="G191" s="4" t="inlineStr"/>
+      <c r="H191" s="4" t="inlineStr"/>
+    </row>
+    <row r="192" ht="22" customHeight="1">
+      <c r="A192" s="2" t="inlineStr"/>
+      <c r="B192" s="2" t="inlineStr"/>
+      <c r="C192" s="3" t="inlineStr"/>
+      <c r="D192" s="2" t="inlineStr"/>
+      <c r="E192" s="2" t="inlineStr"/>
+      <c r="F192" s="2" t="inlineStr"/>
+      <c r="G192" s="2" t="inlineStr"/>
+      <c r="H192" s="2" t="inlineStr"/>
+    </row>
+    <row r="193" ht="22" customHeight="1">
+      <c r="A193" s="4" t="inlineStr"/>
+      <c r="B193" s="4" t="inlineStr"/>
+      <c r="C193" s="5" t="inlineStr"/>
+      <c r="D193" s="4" t="inlineStr"/>
+      <c r="E193" s="4" t="inlineStr"/>
+      <c r="F193" s="4" t="inlineStr"/>
+      <c r="G193" s="4" t="inlineStr"/>
+      <c r="H193" s="4" t="inlineStr"/>
+    </row>
+    <row r="194" ht="22" customHeight="1">
+      <c r="A194" s="2" t="inlineStr"/>
+      <c r="B194" s="2" t="inlineStr"/>
+      <c r="C194" s="3" t="inlineStr"/>
+      <c r="D194" s="2" t="inlineStr"/>
+      <c r="E194" s="2" t="inlineStr"/>
+      <c r="F194" s="2" t="inlineStr"/>
+      <c r="G194" s="2" t="inlineStr"/>
+      <c r="H194" s="2" t="inlineStr"/>
+    </row>
+    <row r="195" ht="22" customHeight="1">
+      <c r="A195" s="4" t="inlineStr"/>
+      <c r="B195" s="4" t="inlineStr"/>
+      <c r="C195" s="5" t="inlineStr"/>
+      <c r="D195" s="4" t="inlineStr"/>
+      <c r="E195" s="4" t="inlineStr"/>
+      <c r="F195" s="4" t="inlineStr"/>
+      <c r="G195" s="4" t="inlineStr"/>
+      <c r="H195" s="4" t="inlineStr"/>
+    </row>
+    <row r="196" ht="22" customHeight="1">
+      <c r="A196" s="2" t="inlineStr"/>
+      <c r="B196" s="2" t="inlineStr"/>
+      <c r="C196" s="3" t="inlineStr"/>
+      <c r="D196" s="2" t="inlineStr"/>
+      <c r="E196" s="2" t="inlineStr"/>
+      <c r="F196" s="2" t="inlineStr"/>
+      <c r="G196" s="2" t="inlineStr"/>
+      <c r="H196" s="2" t="inlineStr"/>
+    </row>
+    <row r="197" ht="22" customHeight="1">
+      <c r="A197" s="4" t="inlineStr"/>
+      <c r="B197" s="4" t="inlineStr"/>
+      <c r="C197" s="5" t="inlineStr"/>
+      <c r="D197" s="4" t="inlineStr"/>
+      <c r="E197" s="4" t="inlineStr"/>
+      <c r="F197" s="4" t="inlineStr"/>
+      <c r="G197" s="4" t="inlineStr"/>
+      <c r="H197" s="4" t="inlineStr"/>
+    </row>
+    <row r="198" ht="22" customHeight="1">
+      <c r="A198" s="2" t="inlineStr"/>
+      <c r="B198" s="2" t="inlineStr"/>
+      <c r="C198" s="3" t="inlineStr"/>
+      <c r="D198" s="2" t="inlineStr"/>
+      <c r="E198" s="2" t="inlineStr"/>
+      <c r="F198" s="2" t="inlineStr"/>
+      <c r="G198" s="2" t="inlineStr"/>
+      <c r="H198" s="2" t="inlineStr"/>
+    </row>
+    <row r="199" ht="22" customHeight="1">
+      <c r="A199" s="4" t="inlineStr"/>
+      <c r="B199" s="4" t="inlineStr"/>
+      <c r="C199" s="5" t="inlineStr"/>
+      <c r="D199" s="4" t="inlineStr"/>
+      <c r="E199" s="4" t="inlineStr"/>
+      <c r="F199" s="4" t="inlineStr"/>
+      <c r="G199" s="4" t="inlineStr"/>
+      <c r="H199" s="4" t="inlineStr"/>
+    </row>
+    <row r="200" ht="22" customHeight="1">
+      <c r="A200" s="2" t="inlineStr"/>
+      <c r="B200" s="2" t="inlineStr"/>
+      <c r="C200" s="3" t="inlineStr"/>
+      <c r="D200" s="2" t="inlineStr"/>
+      <c r="E200" s="2" t="inlineStr"/>
+      <c r="F200" s="2" t="inlineStr"/>
+      <c r="G200" s="2" t="inlineStr"/>
+      <c r="H200" s="2" t="inlineStr"/>
+    </row>
+    <row r="201" ht="22" customHeight="1">
+      <c r="A201" s="4" t="inlineStr"/>
+      <c r="B201" s="4" t="inlineStr"/>
+      <c r="C201" s="5" t="inlineStr"/>
+      <c r="D201" s="4" t="inlineStr"/>
+      <c r="E201" s="4" t="inlineStr"/>
+      <c r="F201" s="4" t="inlineStr"/>
+      <c r="G201" s="4" t="inlineStr"/>
+      <c r="H201" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1069,10 +2569,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1097,7 +2597,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>วัตถุดิบ</t>
+          <t>ค่าแก๊ส</t>
         </is>
       </c>
       <c r="B2" s="8">
@@ -1112,7 +2612,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>ค่าแพ็กเกจจิ้ง</t>
+          <t>ค่าน้ำแข็ง</t>
         </is>
       </c>
       <c r="B3" s="11">
@@ -1127,7 +2627,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>ค่าสาธารณูปโภค</t>
+          <t>ค่าไก่ทอด</t>
         </is>
       </c>
       <c r="B4" s="8">
@@ -1142,7 +2642,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>ค่าขนส่ง</t>
+          <t>ค่าไก่</t>
         </is>
       </c>
       <c r="B5" s="11">
@@ -1157,7 +2657,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>ค่าแรง/เงินเดือน</t>
+          <t>ค่าหมู</t>
         </is>
       </c>
       <c r="B6" s="8">
@@ -1172,7 +2672,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>ค่าเช่า</t>
+          <t>ค่าข้าว</t>
         </is>
       </c>
       <c r="B7" s="11">
@@ -1187,30 +2687,165 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
+          <t>ค่าผัก</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>COUNTIF('Master Data'!B:B,A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="9">
+        <f>SUMIF('Master Data'!B:B,A8,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>ค่าเครื่องปรุงฯ</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>COUNTIF('Master Data'!B:B,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="12">
+        <f>SUMIF('Master Data'!B:B,A9,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>วัตถุดิบ อื่นๆ</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>COUNTIF('Master Data'!B:B,A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="9">
+        <f>SUMIF('Master Data'!B:B,A10,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>ค่าแพ็กเกจจิ้ง</t>
+        </is>
+      </c>
+      <c r="B11" s="11">
+        <f>COUNTIF('Master Data'!B:B,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="12">
+        <f>SUMIF('Master Data'!B:B,A11,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>ค่าขนส่ง</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>COUNTIF('Master Data'!B:B,A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="9">
+        <f>SUMIF('Master Data'!B:B,A12,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>ค่าเดินทาง</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>COUNTIF('Master Data'!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="12">
+        <f>SUMIF('Master Data'!B:B,A13,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>ค่าแรง/เงินเดือน</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>COUNTIF('Master Data'!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="9">
+        <f>SUMIF('Master Data'!B:B,A14,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>ค่าทดลองเมนูอาหาร</t>
+        </is>
+      </c>
+      <c r="B15" s="11">
+        <f>COUNTIF('Master Data'!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="12">
+        <f>SUMIF('Master Data'!B:B,A15,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>ค่าอุปกรณ์/วัสดุสิ้นเปลือง</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>COUNTIF('Master Data'!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="9">
+        <f>SUMIF('Master Data'!B:B,A16,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
           <t>อื่นๆ</t>
         </is>
       </c>
-      <c r="B8" s="8">
-        <f>COUNTIF('Master Data'!B:B,A8)</f>
-        <v/>
-      </c>
-      <c r="C8" s="9">
-        <f>SUMIF('Master Data'!B:B,A8,'Master Data'!C:C)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="B17" s="11">
+        <f>COUNTIF('Master Data'!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="C17" s="12">
+        <f>SUMIF('Master Data'!B:B,A17,'Master Data'!C:C)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>รวมทั้งหมด</t>
         </is>
       </c>
-      <c r="B9" s="14">
-        <f>SUM(B2:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="15">
-        <f>SUM(C2:C8)</f>
+      <c r="B18" s="14">
+        <f>SUM(B2:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>SUM(C2:C17)</f>
         <v/>
       </c>
     </row>

</xml_diff>